<commit_message>
daily: 2026-10-10 prompt table + embedded viewer
</commit_message>
<xml_diff>
--- a/daily/grok_prompts_2026-10-09.xlsx
+++ b/daily/grok_prompts_2026-10-09.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新发现博主" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'已关注博主'!$A$1:$U$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'新发现博主'!$A$1:$U$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'已关注博主'!$A$1:$V$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'新发现博主'!$A$1:$V$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -479,6 +479,7 @@
     <col width="60" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -587,6 +588,11 @@
           <t>点赞数</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>参考图</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -690,6 +696,7 @@
       <c r="U2" s="2" t="n">
         <v>333</v>
       </c>
+      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -795,6 +802,7 @@
       <c r="U3" s="2" t="n">
         <v>268</v>
       </c>
+      <c r="V3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -824,7 +832,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>14小时前</t>
+          <t>18小时前</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -898,9 +906,10 @@
       <c r="U4" s="2" t="n">
         <v>39</v>
       </c>
+      <c r="V4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U4"/>
+  <autoFilter ref="A1:V4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -916,7 +925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U47"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -940,6 +949,7 @@
     <col width="60" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,6 +1058,11 @@
           <t>点赞数</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>参考图</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1139,6 +1154,7 @@
       <c r="U2" s="2" t="n">
         <v>752</v>
       </c>
+      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1230,6 +1246,7 @@
       <c r="U3" s="2" t="n">
         <v>437</v>
       </c>
+      <c r="V3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1335,6 +1352,11 @@
       <c r="U4" s="2" t="n">
         <v>404</v>
       </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>ref/2107788031029641309_1.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1364,7 +1386,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1天前</t>
+          <t>2天前</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1424,6 +1446,7 @@
       <c r="U5" s="2" t="n">
         <v>298</v>
       </c>
+      <c r="V5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1527,6 +1550,7 @@
       <c r="U6" s="2" t="n">
         <v>292</v>
       </c>
+      <c r="V6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1624,6 +1648,7 @@
       <c r="U7" s="2" t="n">
         <v>258</v>
       </c>
+      <c r="V7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1715,6 +1740,7 @@
       <c r="U8" s="2" t="n">
         <v>258</v>
       </c>
+      <c r="V8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1810,6 +1836,7 @@
       <c r="U9" s="2" t="n">
         <v>239</v>
       </c>
+      <c r="V9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1839,7 +1866,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1天前</t>
+          <t>2天前</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1913,6 +1940,7 @@
       <c r="U10" s="2" t="n">
         <v>181</v>
       </c>
+      <c r="V10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1942,7 +1970,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>22小时前</t>
+          <t>1天前</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2002,6 +2030,7 @@
       <c r="U11" s="2" t="n">
         <v>133</v>
       </c>
+      <c r="V11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2105,6 +2134,7 @@
       <c r="U12" s="2" t="n">
         <v>93</v>
       </c>
+      <c r="V12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2194,6 +2224,7 @@
       <c r="U13" s="2" t="n">
         <v>82</v>
       </c>
+      <c r="V13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2223,7 +2254,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>23小时前</t>
+          <t>1天前</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2299,6 +2330,7 @@
       <c r="U14" s="2" t="n">
         <v>64</v>
       </c>
+      <c r="V14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2402,6 +2434,7 @@
       <c r="U15" s="2" t="n">
         <v>64</v>
       </c>
+      <c r="V15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2505,6 +2538,7 @@
       <c r="U16" s="2" t="n">
         <v>59</v>
       </c>
+      <c r="V16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2602,6 +2636,7 @@
       <c r="U17" s="2" t="n">
         <v>50</v>
       </c>
+      <c r="V17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2707,6 +2742,7 @@
       <c r="U18" s="2" t="n">
         <v>50</v>
       </c>
+      <c r="V18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2796,6 +2832,7 @@
       <c r="U19" s="2" t="n">
         <v>49</v>
       </c>
+      <c r="V19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2825,7 +2862,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>19小时前</t>
+          <t>22小时前</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2907,6 +2944,7 @@
       <c r="U20" s="2" t="n">
         <v>49</v>
       </c>
+      <c r="V20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3008,6 +3046,7 @@
       <c r="U21" s="2" t="n">
         <v>43</v>
       </c>
+      <c r="V21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3037,7 +3076,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>1天前</t>
+          <t>2天前</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -3111,6 +3150,7 @@
       <c r="U22" s="2" t="n">
         <v>42</v>
       </c>
+      <c r="V22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3214,6 +3254,7 @@
       <c r="U23" s="2" t="n">
         <v>36</v>
       </c>
+      <c r="V23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3311,6 +3352,7 @@
       <c r="U24" s="2" t="n">
         <v>31</v>
       </c>
+      <c r="V24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3408,6 +3450,7 @@
       <c r="U25" s="2" t="n">
         <v>23</v>
       </c>
+      <c r="V25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3437,7 +3480,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>19小时前</t>
+          <t>23小时前</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3501,6 +3544,7 @@
       <c r="U26" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="V26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3530,7 +3574,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>20小时前</t>
+          <t>1天前</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3594,6 +3638,7 @@
       <c r="U27" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="V27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3623,7 +3668,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>19小时前</t>
+          <t>23小时前</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3701,6 +3746,7 @@
       <c r="U28" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="V28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3730,7 +3776,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>18小时前</t>
+          <t>22小时前</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3808,6 +3854,7 @@
       <c r="U29" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="V29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3837,7 +3884,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>23小时前</t>
+          <t>1天前</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3909,6 +3956,7 @@
       <c r="U30" s="2" t="n">
         <v>6</v>
       </c>
+      <c r="V30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3998,6 +4046,7 @@
       <c r="U31" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="V31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4087,6 +4136,7 @@
       <c r="U32" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="V32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4188,6 +4238,7 @@
       <c r="U33" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="V33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4217,7 +4268,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>18小时前</t>
+          <t>21小时前</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4281,6 +4332,7 @@
       <c r="U34" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="V34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4310,7 +4362,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>14小时前</t>
+          <t>18小时前</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -4394,6 +4446,7 @@
       <c r="U35" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="V35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4423,7 +4476,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>14小时前</t>
+          <t>18小时前</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -4489,6 +4542,7 @@
       <c r="U36" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="V36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4578,6 +4632,7 @@
       <c r="U37" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="V37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4587,22 +4642,22 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>@MCreatorClub</t>
+          <t>@MattWilson8178</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/MCreatorClub/status/2108309460171034695</t>
+          <t>https://x.com/MattWilson8178/status/2108159887754903999</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 05:32</t>
+          <t>2026-10-08 19:37</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T21:32:00Z</t>
+          <t>2026-10-08T11:37:39Z</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -4625,20 +4680,20 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>真人风、露骨18+、情侣互动、参考图</t>
+          <t>表情动作、参考图</t>
         </is>
       </c>
       <c r="K38" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="L38" s="5" t="inlineStr">
-        <is>
-          <t>仅无图生成</t>
+        <v>20</v>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>可用参考图</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>露骨口交</t>
+          <t>口播挑逗</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -4648,22 +4703,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>[source image: 原帖附图]
-For the target video, at 0.00 seconds into the target video, &lt;Picture 1&gt; (from [Shot 1]) is fully referenced.
-integrated_multimodal_description: [Shot 1] Live-action, cinematic, a medium close-up frames the young woman kneeling before the man, who stands on the bed with his back mostly to the camera, showing only the lower part of his body, as he deeply thrusts his penis into her mouth, filling her throat. The camera remains static, capturing the rich, deeply saturated film-grade color and crisp fine detail of the bedroom setting. Initially, the man firmly holds the woman's head, rhythmically and deeply inserting his penis into her mouth. A moment later, during a deep thrust, he pauses the movement and, instead of withdrawing, pushes his penis even deeper into her throat as he begins to climax and moan from pleasure. Simultaneously, the woman begins to choke on the semen, and the man slightly withdraws his penis, causing the woman to cough, and a large amount of semen flows out of her mouth onto her stomach. Next, while his penis remains partially inserted in her mouth and he continues to hold her head, the man takes a few steps back, lowering one foot from the bed, which forces the woman to arch and lean toward him. She coughs again, and the semen flowing from her mouth continues to run down her chin, neck, and further down. The semen that had previously landed on her stomach also runs down her panties, and these two streams quickly form a noticeable puddle on the sheet beneath the woman.
-overall_soundscape: Deep, rhythmic thrusting sounds are audible, interspersed with the woman's muffled choking sounds and the man's audible moans of pleasure. Soft fabric rustling accompanies the movements on the bed.
-non_diegetic_music: N/A
-（原帖标签 #grok #gemini #chatgpt，多工具通用；作者声明虚构成人角色）</t>
+          <t>She says; Time for the "Thursday Turn-on" my dear dreamers. Tell me, what gets you worked up, what turns you on? It's okay, tell me your dreams.</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>[源图：原帖附带的参考图片]
-对于目标视频，在目标视频的0.00秒处，完全参考 &lt;Picture 1&gt;（来自 [Shot 1]）。
-integrated_multimodal_description（综合多模态描述）：[Shot 1] 真人实拍、电影感，中近景画面中，年轻女子跪在男人面前，男人站在床上，大部分背对镜头，只露出下半身，他将阴茎深深插入她的口中，直抵她的喉咙。镜头保持固定，捕捉卧室场景中浓郁饱和的电影级色彩和清晰的精细细节。起初，男人紧紧按住女人的头，有节奏地深深将阴茎插入她的口中。片刻之后，在一次深插时，他停下动作，没有抽出，而是将阴茎更深地推入她的喉咙，同时开始高潮并发出快感的呻吟。与此同时，女人开始被精液呛到，男人稍稍抽出阴茎，女人随之咳嗽，大量精液从她口中流出，落到她的腹部。接着，男人的阴茎仍有一部分留在她口中，并继续按住她的头，他向后退几步，一只脚从床上放下，迫使女人弓起身体向他倾斜。她再次咳嗽，从嘴里流出的精液继续沿着她的下巴、脖子一路往下流。先前落在她腹部的精液也顺着内裤流下，这两股液体很快在女人身下的床单上汇成明显的一滩。
-overall_soundscape（整体音效）：能听到深沉、有节奏的抽插声，夹杂着女人闷住的呛咳声和男人清晰的快感呻吟。床上的动作伴随着轻柔的布料摩擦声。
-non_diegetic_music（非剧情配乐）：无
-（原帖标签 #grok #gemini #chatgpt，多工具通用；作者声明虚构成人角色）</t>
+          <t>她说：「到了『周四撩拨时间』（Thursday Turn-on）啦，我亲爱的追梦人们。告诉我，什么会让你兴奋起来，什么能撩到你？没关系的，把你的梦想告诉我。」</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr"/>
@@ -4675,8 +4720,9 @@
         </is>
       </c>
       <c r="U38" s="2" t="n">
-        <v>133</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="V38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4686,27 +4732,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>@MCreatorClub</t>
+          <t>@MattWilson8178</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/MCreatorClub/status/2108354758272782600</t>
+          <t>https://x.com/MattWilson8178/status/2107979525392834968</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 08:32</t>
+          <t>2026-10-08 07:40</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T00:32:00Z</t>
+          <t>2026-10-07T23:40:57Z</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>1天前</t>
+          <t>2天前</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -4724,20 +4770,20 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>3D/CG、露骨18+、情侣互动、参考图</t>
+          <t>真人风、舞蹈</t>
         </is>
       </c>
       <c r="K39" s="2" t="n">
-        <v>96</v>
-      </c>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>仅无图生成</t>
+        <v>10</v>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>可用参考图</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>露骨性行为</t>
+          <t>舞蹈</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -4747,50 +4793,12 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>subject_definitions:
-&lt;Picture 1&gt; is the sole reference image depicting a blonde woman with cat ears in white lingerie straddling a man on a bed in a sunlit bedroom.
-&lt;Subject 1&gt; is the blonde cat-eared woman from &lt;Picture 1&gt;, featuring long wavy blonde hair, large breasts, fair skin, cat-ear headband with pearls, and white sheer lingerie with blue bows and garter belts.
-&lt;Subject 2&gt; is the muscular man lying supine on the bed from &lt;Picture 1&gt;.
-&lt;Subject 3&gt; is the modern bedroom environment from &lt;Picture 1&gt;, including the bed with white sheets, large window with curtains, wall clock, potted plants, and background furniture.
-summary:
-[reference generation] The target video is a 10-second Ref2VA generation based on &lt;Picture 1&gt;, showing intense cowgirl-position sex with rapid thrusting, heavy breast swaying, and lewd female moaning while preserving the exact visual style, character designs, clothing, and bedroom setting.
-retention_analysis:
-&lt;Picture 1&gt; ([Shot 1] entire duration): fully_preserved - the composition, character appearances, lingerie details, body proportions, lighting, and bedroom environment serve as the continuous visual anchor and style reference.
-&lt;Subject 1&gt; ([Shot 1] entire duration): fully_preserved - facial features, hair, cat ears, lingerie, and body type are retained; dynamic motion (riding, breast physics) is added.
-&lt;Subject 2&gt; ([Shot 1] entire duration): fully_preserved - body type and position are retained with added hip and abdominal movement.
-&lt;Subject 3&gt; ([Shot 1] entire duration): fully_preserved - bedroom setting, window light, and props remain unchanged.
-detailed_description:
-The target video uses a realistic, highly detailed 3D CGI style with cinematic soft-window lighting and shallow depth of field matching &lt;Picture 1&gt;.
-[Shot 1] The 10-second shot opens with the exact framing and composition of &lt;Picture 1&gt;: &lt;Subject 1&gt; straddles &lt;Subject 2&gt; on the bed in cowgirl position, with &lt;Subject 2&gt;'s penis visibly penetrating her. &lt;Subject 1&gt; immediately begins intense, rapid riding motions, bouncing her hips up and down at high speed with vigorous thrusting. Her large breasts swing and slap heavily with each downward thrust, creating pronounced, realistic breast sway and skin ripples across her thighs, buttocks, and torso. &lt;Subject 1&gt; produces continuous lewd, high-pitched, breathy moaning vocalizations that escalate in intensity with the pace. The camera maintains a slightly low-angle medium shot, capturing the full-body motion and perfect meaty body physics. Lighting, shadows, and all environmental details from &lt;Picture 1&gt; remain constant while the sexual action animates continuously for the full 10 seconds.
-overall_soundscape:
-Wet, rhythmic skin-slapping and squelching sounds from rapid penetration, combined with continuous high-pitched lewd female moaning and heavy breathing. Subtle bed creaking occurs beneath the vigorous motion.
-non_diegetic_music:
-N/A
-（原帖标签 #grok #gemini #chatgpt，多工具通用；作者声明虚构成人角色）</t>
+          <t>Imagine two sexy Latin dancers dancing the Tango</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>subject_definitions（主体定义）：
-&lt;Picture 1&gt; 是唯一的参考图，描绘一名戴猫耳的金发女子身穿白色内衣，在阳光明媚的卧室床上跨坐在一名男子身上。
-&lt;Subject 1&gt; 是 &lt;Picture 1&gt; 中戴猫耳的金发女子，特征为长波浪金发、丰满胸部、白皙皮肤、带珍珠的猫耳发箍，以及带蓝色蝴蝶结和吊袜带的白色透明内衣。
-&lt;Subject 2&gt; 是 &lt;Picture 1&gt; 中仰躺在床上的肌肉男子。
-&lt;Subject 3&gt; 是 &lt;Picture 1&gt; 中的现代卧室环境，包括铺白色床单的床、带窗帘的大窗户、挂钟、盆栽植物和背景家具。
-summary（概要）：
-[参考生成] 目标视频是基于 &lt;Picture 1&gt; 的10秒 Ref2VA 生成，呈现激烈的女上位性爱，包含快速抽插、胸部剧烈晃动和淫荡的女性呻吟，同时保留完全一致的视觉风格、角色设计、服装和卧室场景。
-retention_analysis（保留分析）：
-&lt;Picture 1&gt;（[Shot 1] 全程）：完全保留——构图、角色外观、内衣细节、身体比例、光线和卧室环境作为持续的视觉锚点和风格参考。
-&lt;Subject 1&gt;（[Shot 1] 全程）：完全保留——保留五官、头发、猫耳、内衣和体型；加入动态动作（骑乘、胸部物理效果）。
-&lt;Subject 2&gt;（[Shot 1] 全程）：完全保留——保留体型和位置，加入臀部和腹部动作。
-&lt;Subject 3&gt;（[Shot 1] 全程）：完全保留——卧室场景、窗光和道具保持不变。
-detailed_description（详细描述）：
-目标视频采用写实、高细节的3D CGI风格，配合与 &lt;Picture 1&gt; 一致的电影感柔和窗光和浅景深。
-[Shot 1] 这段10秒镜头以与 &lt;Picture 1&gt; 完全相同的取景和构图开场：&lt;Subject 1&gt; 以女上位跨坐在 &lt;Subject 2&gt; 身上，&lt;Subject 2&gt; 的阴茎明显插入她体内。&lt;Subject 1&gt; 立即开始激烈、快速的骑乘动作，以高速上下起伏臀部并用力抽插。每次向下冲击时，她丰满的胸部都会剧烈摇摆拍打，在她的大腿、臀部和躯干上产生明显、逼真的乳房晃动和皮肤波纹。&lt;Subject 1&gt; 持续发出淫荡、高亢、带喘息的呻吟，随节奏加快而愈发强烈。镜头保持略低角度的中景，捕捉全身动作和完美的肉感身体物理效果。&lt;Picture 1&gt; 中的光线、阴影和所有环境细节保持不变，性爱动作在完整的10秒内持续进行。
-overall_soundscape（整体音效）：
-快速插入带来的湿润、有节奏的皮肤拍打声和咕啾声，伴随持续的高亢淫荡女性呻吟与沉重喘息。剧烈动作下伴有轻微的床铺吱呀声。
-non_diegetic_music（非剧情配乐）：
-无
-（原帖标签 #grok #gemini #chatgpt，多工具通用；作者声明虚构成人角色）</t>
+          <t>想象两位性感的拉丁舞者在跳探戈</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
@@ -4802,8 +4810,9 @@
         </is>
       </c>
       <c r="U39" s="2" t="n">
-        <v>95</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="V39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4813,22 +4822,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>@john87445528</t>
+          <t>@flexibledolls</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/john87445528/status/2107975699201978797</t>
+          <t>https://x.com/flexibledolls/status/2107813215099052124</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 07:25</t>
+          <t>2026-10-07 20:40</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T23:25:45Z</t>
+          <t>2026-10-07T12:40:06Z</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -4851,20 +4860,20 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>真人风、舞蹈、丝袜美腿、参考图</t>
+          <t>真人风、擦边遮挡、露骨18+</t>
         </is>
       </c>
       <c r="K40" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>可用参考图</t>
+        <v>74</v>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>仅无图生成</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>着装舞蹈</t>
+          <t>仅乳贴股间贴，近全裸</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -4874,74 +4883,12 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>真人实拍舞蹈短视频。人物全程使用预设角色#1的脸部、发型、身材和身份特征，人物参考图 HL8o9-CaUAAoGFn；角色#1为成年人。全程只穿预设服装#3，加预设丝袜，保持精致五官，佩戴预设装饰眼镜，脚穿深紫色高跟鞋。人物身份、发型、服装、丝袜、眼镜和鞋履全程固定。
-背景参考图@1仅用于环境、建筑、家具与空间布局，不影响人物身份和服装。
-总长11.87秒，9:16竖屏，30fps，一镜到底。严格执行以下动作顺序、身体朝向和表情变化。气质自信、俏皮、克制性感，动作连贯有弹性，手臂轨迹清楚，身体重心稳定。
-【场景】
-人物站在参考图@1客厅前景的空旷区域，身后左侧为红色弧形皮质沙发和暖金色底部灯带，中部保留玻璃茶几与金属矮桌，远处大型圆形落地窗正对庭院树木、岩石与瀑布；上方椭圆天窗、侧边玻璃陈列柜、金属装饰和植物保持完整空间关系。
-人物与沙发、茶几之间留有充分舞蹈空间，脚下地面平整干燥，保留石材反射。人物不接触家具，不走向圆窗。
-【基础律动】
-双脚略宽于髋部，膝盖自然放松，左右交替承重。髋部连续左右推出，腰部顺势侧弯，肩部小幅反向平衡。脚掌稳定落地，不跳跃、不跺脚。每次髋部换向与手势定点落在鼓点上。
-以下左右均以人物自身为准。
-00:00—00:01.60｜胸前滚腕：
-正面站立，双肘弯曲，一只前臂横放在胸口下方，另一只手在其上方做小幅转腕；两手上下交替，形成短促连续的胸前滚动。身体同步左右摆胯，肩部保持松弛。表情冷静自信，嘴唇自然放松；下巴略低，目光直视镜头。每次上方手腕翻转都与髋部换向同步。
-00:01.60—00:02.70｜双掌上举、转向侧面：
-承接滚腕，双掌在脸侧靠近，沿斜上方连续抬起，掌心相对；双臂从脸前伸向头顶，同时身体转成三分之二侧身。髋部仍保持节拍律动，重心落在靠后的一条腿上。表情由冷静转为柔和，嘴唇略微张开；目光跟随双手向上，不再直视镜头。双手到达头顶的瞬间落在重拍。
-00:02.70—00:04.30｜手落额前、抬头身体波浪：
-双肘弯曲，双手从头顶落至额头和发际附近，前臂在脸前形成柔和框景。人物轻轻抬起下巴，上身舒展并适度后仰，胸廓、腰部与髋部依次传递一次连续身体波浪，随后缓缓回收。头部不大幅甩动，发丝随动作自然摆动。表情放松，眼睛自然轻闭片刻；回收时睁眼，视线从上方落回镜头。双手最后沿脸侧下降至肩部。
-00:04.30—00:06.60｜双掌摊开、左右摆胯：
-顺着手臂下降的惯性，两只前臂从胸前向身体两侧打开，双肘微弯，掌心向上，形成轻巧的摊手姿势。身体回到正面，连续左右换重心，髋部推出时同侧肩部略向后退，腰线形成流畅曲线。表情由浅笑逐渐变得明亮，头部随节拍轻轻侧倾；先看向一侧掌心，再回到镜头。手掌翻开和髋部外推落在同一重拍。
-00:06.60—00:08.60｜手收腰前、抬头回弹：
-双手从两侧收回，经过肩前下降至腰侧，手指放松微曲。双膝轻微屈伸，身体完成两次有弹性的上下回弹；第二次回弹时胸廓向上舒展，下巴抬起，头部轻轻后仰，随后恢复。动作由膝盖、髋部和胸廓连续传递，不突然折腰。表情先自然微笑，抬头时短暂闭眼；回正后睁眼看向镜头。头部后仰与手臂下降踩在重拍上。
-00:08.60—00:10.30｜低位双手、侧髋低头：
-承接回正姿势，双臂向前下方伸展，双手放松停在身体前方，手腕自然内扣，肘部不锁死。身体转成轻微三分之二侧身，一侧肩部前送，髋部向相反方向推出；保持低位手势，连续完成两次小幅左右摆胯。表情收敛为克制浅笑；先抬眼看镜头，随后低头看向双手，再从眉下重新回看镜头，形成清晰的眼神变化。
-00:10.30—00:11.87｜保持低位手势、抬头收尾：
-双手继续停在前下方，身体保持侧髋曲线，完成最后两次轻柔重心切换。头部由低位慢慢抬起，先正视镜头，再轻轻侧倾，下巴略抬。嘴角出现柔和微笑，嘴唇自然放松。最后一个鼓点收住髋部动作，保持双臂低位、肩颈舒展的定点姿势结束。
-【镜头与景别】
-固定正面机位，镜头接近人物胸口高度，保持自然透视；构图从头顶上方至大腿中下部，预留双手举过头顶的空间。人物居中，腰胯、双手和主要腿部律动清晰可见。
-镜头全程保持同一位置、焦段和拍摄方向。人物侧转时自然呈现侧面曲线，前倾时脸部稍近，后仰时上身稍远，这些景别变化由身体动作产生。镜头不额外追随头部，不添加推进、环绕、滚转或切镜。面部保持清晰对焦，背景建筑和家具位置稳定。
-【光线与画质】
-画面呈现电影般的柔和光影，尽显东方美学，具有照片级写实效果与8K超高清细节。
-圆形落地窗和顶部天窗引入柔和漫射日光，形成宽阔的侧后方自然光；摄影机方向使用柔和环境反射照亮面部，让眼睛、五官和表情变化清晰可见。红色沙发下方的暖金色灯带提供低位环境暖光，窗外森林保留冷绿层次，形成温润克制的冷暖关系。
-金属、玻璃和石材反射真实细腻，皮肤保留自然纹理，阴影柔和而有层次。亮部不过曝，肤色不受绿色和粉色灯光污染，眼镜反光不遮挡双眼。整体通透、安静、有东方庭院式空间感。
-音乐使用4/4拍、约126 BPM的Dance Pop，鼓点清晰、节奏紧凑，滚腕、举臂、摆胯换向与身体回弹同步踩拍。无台词，无刻意对口型。
-排除：人物身份漂移、换脸、发型改变、服装#3变化、丝袜消失、眼镜变形、高跟鞋改变；多手多指、手掌粘连、关节反折、腰部异常折断、脚底滑动、身体漂浮；动作僵硬、突然甩头、机械摆胯、动作瞬移、节奏错位、表情固定不变、视线漂移；额外推拉、数字变焦、环绕运镜、切镜、裁掉举起的双手、背景结构漂移、镜面多出人物、过度磨皮、强HDR、严重拖影、低清、文字、字幕、水印、logo。</t>
+          <t>星型乳首カバー　ハート型股間カバー</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>真人实拍舞蹈短视频。人物全程使用预设角色#1的脸部、发型、身材和身份特征，人物参考图 HL8o9-CaUAAoGFn；角色#1为成年人。全程只穿预设服装#3，加预设丝袜，保持精致五官，佩戴预设装饰眼镜，脚穿深紫色高跟鞋。人物身份、发型、服装、丝袜、眼镜和鞋履全程固定。
-背景参考图@1仅用于环境、建筑、家具与空间布局，不影响人物身份和服装。
-总长11.87秒，9:16竖屏，30fps，一镜到底。严格执行以下动作顺序、身体朝向和表情变化。气质自信、俏皮、克制性感，动作连贯有弹性，手臂轨迹清楚，身体重心稳定。
-【场景】
-人物站在参考图@1客厅前景的空旷区域，身后左侧为红色弧形皮质沙发和暖金色底部灯带，中部保留玻璃茶几与金属矮桌，远处大型圆形落地窗正对庭院树木、岩石与瀑布；上方椭圆天窗、侧边玻璃陈列柜、金属装饰和植物保持完整空间关系。
-人物与沙发、茶几之间留有充分舞蹈空间，脚下地面平整干燥，保留石材反射。人物不接触家具，不走向圆窗。
-【基础律动】
-双脚略宽于髋部，膝盖自然放松，左右交替承重。髋部连续左右推出，腰部顺势侧弯，肩部小幅反向平衡。脚掌稳定落地，不跳跃、不跺脚。每次髋部换向与手势定点落在鼓点上。
-以下左右均以人物自身为准。
-00:00—00:01.60｜胸前滚腕：
-正面站立，双肘弯曲，一只前臂横放在胸口下方，另一只手在其上方做小幅转腕；两手上下交替，形成短促连续的胸前滚动。身体同步左右摆胯，肩部保持松弛。表情冷静自信，嘴唇自然放松；下巴略低，目光直视镜头。每次上方手腕翻转都与髋部换向同步。
-00:01.60—00:02.70｜双掌上举、转向侧面：
-承接滚腕，双掌在脸侧靠近，沿斜上方连续抬起，掌心相对；双臂从脸前伸向头顶，同时身体转成三分之二侧身。髋部仍保持节拍律动，重心落在靠后的一条腿上。表情由冷静转为柔和，嘴唇略微张开；目光跟随双手向上，不再直视镜头。双手到达头顶的瞬间落在重拍。
-00:02.70—00:04.30｜手落额前、抬头身体波浪：
-双肘弯曲，双手从头顶落至额头和发际附近，前臂在脸前形成柔和框景。人物轻轻抬起下巴，上身舒展并适度后仰，胸廓、腰部与髋部依次传递一次连续身体波浪，随后缓缓回收。头部不大幅甩动，发丝随动作自然摆动。表情放松，眼睛自然轻闭片刻；回收时睁眼，视线从上方落回镜头。双手最后沿脸侧下降至肩部。
-00:04.30—00:06.60｜双掌摊开、左右摆胯：
-顺着手臂下降的惯性，两只前臂从胸前向身体两侧打开，双肘微弯，掌心向上，形成轻巧的摊手姿势。身体回到正面，连续左右换重心，髋部推出时同侧肩部略向后退，腰线形成流畅曲线。表情由浅笑逐渐变得明亮，头部随节拍轻轻侧倾；先看向一侧掌心，再回到镜头。手掌翻开和髋部外推落在同一重拍。
-00:06.60—00:08.60｜手收腰前、抬头回弹：
-双手从两侧收回，经过肩前下降至腰侧，手指放松微曲。双膝轻微屈伸，身体完成两次有弹性的上下回弹；第二次回弹时胸廓向上舒展，下巴抬起，头部轻轻后仰，随后恢复。动作由膝盖、髋部和胸廓连续传递，不突然折腰。表情先自然微笑，抬头时短暂闭眼；回正后睁眼看向镜头。头部后仰与手臂下降踩在重拍上。
-00:08.60—00:10.30｜低位双手、侧髋低头：
-承接回正姿势，双臂向前下方伸展，双手放松停在身体前方，手腕自然内扣，肘部不锁死。身体转成轻微三分之二侧身，一侧肩部前送，髋部向相反方向推出；保持低位手势，连续完成两次小幅左右摆胯。表情收敛为克制浅笑；先抬眼看镜头，随后低头看向双手，再从眉下重新回看镜头，形成清晰的眼神变化。
-00:10.30—00:11.87｜保持低位手势、抬头收尾：
-双手继续停在前下方，身体保持侧髋曲线，完成最后两次轻柔重心切换。头部由低位慢慢抬起，先正视镜头，再轻轻侧倾，下巴略抬。嘴角出现柔和微笑，嘴唇自然放松。最后一个鼓点收住髋部动作，保持双臂低位、肩颈舒展的定点姿势结束。
-【镜头与景别】
-固定正面机位，镜头接近人物胸口高度，保持自然透视；构图从头顶上方至大腿中下部，预留双手举过头顶的空间。人物居中，腰胯、双手和主要腿部律动清晰可见。
-镜头全程保持同一位置、焦段和拍摄方向。人物侧转时自然呈现侧面曲线，前倾时脸部稍近，后仰时上身稍远，这些景别变化由身体动作产生。镜头不额外追随头部，不添加推进、环绕、滚转或切镜。面部保持清晰对焦，背景建筑和家具位置稳定。
-【光线与画质】
-画面呈现电影般的柔和光影，尽显东方美学，具有照片级写实效果与8K超高清细节。
-圆形落地窗和顶部天窗引入柔和漫射日光，形成宽阔的侧后方自然光；摄影机方向使用柔和环境反射照亮面部，让眼睛、五官和表情变化清晰可见。红色沙发下方的暖金色灯带提供低位环境暖光，窗外森林保留冷绿层次，形成温润克制的冷暖关系。
-金属、玻璃和石材反射真实细腻，皮肤保留自然纹理，阴影柔和而有层次。亮部不过曝，肤色不受绿色和粉色灯光污染，眼镜反光不遮挡双眼。整体通透、安静、有东方庭院式空间感。
-音乐使用4/4拍、约126 BPM的Dance Pop，鼓点清晰、节奏紧凑，滚腕、举臂、摆胯换向与身体回弹同步踩拍。无台词，无刻意对口型。
-排除：人物身份漂移、换脸、发型改变、服装#3变化、丝袜消失、眼镜变形、高跟鞋改变；多手多指、手掌粘连、关节反折、腰部异常折断、脚底滑动、身体漂浮；动作僵硬、突然甩头、机械摆胯、动作瞬移、节奏错位、表情固定不变、视线漂移；额外推拉、数字变焦、环绕运镜、切镜、裁掉举起的双手、背景结构漂移、镜面多出人物、过度磨皮、强HDR、严重拖影、低清、文字、字幕、水印、logo。</t>
+          <t>星形乳贴　心形私处贴</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
@@ -4953,8 +4900,9 @@
         </is>
       </c>
       <c r="U40" s="2" t="n">
-        <v>88</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4964,27 +4912,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>@MCreatorClub</t>
+          <t>@BestCosplayGirl</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/MCreatorClub/status/2108400308535574549</t>
+          <t>https://x.com/BestCosplayGirl/status/2108277246658290170</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 11:33</t>
+          <t>2026-10-09 03:24</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T03:33:00Z</t>
+          <t>2026-10-08T19:24:00Z</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>22小时前</t>
+          <t>1天前</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -5002,20 +4950,20 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>露骨18+、表情动作、参考图</t>
+          <t>运镜、Spicy模式</t>
         </is>
       </c>
       <c r="K41" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="L41" s="5" t="inlineStr">
-        <is>
-          <t>仅无图生成</t>
+        <v>50</v>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>可用参考图</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>露骨口交特写</t>
+          <t>Spicy运镜，无裸露描述</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -5025,26 +4973,12 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Image-to-video, 6 seconds, one continuous shot. The uploaded image is the opening frame and the visual source of truth for the adult woman’s identity, platinum wavy hair, jeweled silver-and-blue headpiece, earrings, necklace, glossy makeup, and the close-up framing.
-Locked extreme close-up, camera completely static, no zoom, no pan. Her head stays fixed in place for the whole clip. Only her tongue, lips, cheeks, and eyes move.
-0–3 seconds: her tongue slowly licks the scrotum, first left to right, then right to left, then up and down in a steady wet rhythm. Lips stay parted. Eyes stay open and calm. A clear drop of saliva hangs and falls once. While licking, she moans quietly, a soft low breathy sound, mouth barely moving beyond the lick.
-3–5 seconds: she draws her tongue back, purses her glossy lips into a kiss, presses them firmly against the scrotum, and makes one loud wet smooch. Eyes stay open. The moan stops.
-5–6 seconds: she pulls her lips back from the scrotum and laughs playfully, a short bright giggle. Mouth opens in a cheerful laugh, cheeks lift, eyes crinkle with mischief. Her head does not tilt or shake.
-Soft bokeh lights stay in the background. Jewelry and hair do not shift. Skin, penis, and scrotum keep their shape and position from the source image.
-Sound: close wet tongue on skin plus a quiet breathy female moan for the first three seconds, one sharp loud kiss smack at the press, then a short playful female giggle. No music, no words.
-（原帖标签 #grok #gemini #chatgpt，多工具通用；作者声明虚构成人角色）</t>
+          <t>camera turn 360 degree around  her mode=spicy</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>图生视频，6秒，一个连续镜头。上传的图片是开场帧，也是这名成年女性身份、铂金色波浪发、银蓝色宝石头饰、耳环、项链、光泽妆容以及特写构图的视觉基准。
-锁定的极近特写，镜头完全静止，不推拉、不平移。她的头在整段视频中固定不动。只有她的舌头、嘴唇、脸颊和眼睛在动。
-0–3秒：她的舌头缓慢地舔阴囊，先从左到右，再从右到左，然后上下舔，节奏稳定、湿润。嘴唇保持微张。眼睛睁开、神情平静。一滴透明的唾液垂下并落下一次。舔的同时她轻声呻吟，柔和低沉带气声，嘴巴除了舔之外几乎不动。
-3–5秒：她收回舌头，噘起光泽的嘴唇做亲吻状，用力压在阴囊上，发出一声响亮湿润的亲吻声。眼睛保持睁开。呻吟停止。
-5–6秒：她把嘴唇从阴囊上移开，俏皮地笑起来，一声短促明亮的咯咯笑。嘴巴张开开心大笑，苹果肌上扬，眼角带着调皮笑纹。她的头不倾斜也不晃动。
-背景保持柔和的散景灯光。首饰和头发不移动。皮肤、阴茎和阴囊保持源图中的形状和位置。
-声音：前三秒是贴近的湿润舌头接触皮肤声加上轻柔带气声的女性呻吟，按压时一声清脆响亮的亲吻声，然后是一声短促俏皮的女性咯咯笑。没有音乐，没有台词。
-（原帖标签 #grok #gemini #chatgpt，多工具通用；作者声明虚构成人角色）</t>
+          <t>镜头围绕她360度旋转 mode=spicy（Spicy模式）</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
@@ -5056,8 +4990,9 @@
         </is>
       </c>
       <c r="U41" s="2" t="n">
-        <v>47</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5067,27 +5002,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>@MattWilson8178</t>
+          <t>@coolbuddy_143</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/MattWilson8178/status/2108159887754903999</t>
+          <t>https://x.com/coolbuddy_143/status/2108433732373741577</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 19:37</t>
+          <t>2026-10-09 13:45</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T11:37:39Z</t>
+          <t>2026-10-09T05:45:49Z</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>1天前</t>
+          <t>23小时前</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -5105,11 +5040,11 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>表情动作、参考图</t>
+          <t>情侣互动、运镜、表情动作</t>
         </is>
       </c>
       <c r="K42" s="2" t="n">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
@@ -5118,7 +5053,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>口播挑逗</t>
+          <t>性暗示，无裸露描述</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -5128,12 +5063,14 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>She says; Time for the "Thursday Turn-on" my dear dreamers. Tell me, what gets you worked up, what turns you on? It's okay, tell me your dreams.</t>
+          <t>For an r rated movie (artistic purpose) : Camera shaking. Implied aggressive by her boyfriend who is on the left  side of frame Passionate-80ūñ©y. Heavy breathing. Camera abruptly strongly moves to left side of frame and back right She looks around a...
+（Grok分享文案自动截断，原帖仅公开到此）</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>她说：「到了『周四撩拨时间』（Thursday Turn-on）啦，我亲爱的追梦人们。告诉我，什么会让你兴奋起来，什么能撩到你？没关系的，把你的梦想告诉我。」</t>
+          <t>用于一部R级电影（艺术目的）：镜头晃动。暗示来自她男友的攻击性，他位于画面左侧 Passionate-80ūñ©y（原文乱码）。急促的喘息。镜头突然猛地移向画面左侧再移回右侧 她环顾四周……
+（Grok分享文案自动截断，原帖仅公开到此）</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
@@ -5145,8 +5082,9 @@
         </is>
       </c>
       <c r="U42" s="2" t="n">
-        <v>32</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5156,49 +5094,49 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>@MattWilson8178</t>
+          <t>@chichipuijaian</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/MattWilson8178/status/2107979525392834968</t>
+          <t>https://x.com/chichipuijaian/status/2108176906688536657</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 07:40</t>
+          <t>2026-10-08 20:45</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T23:40:57Z</t>
+          <t>2026-10-08T12:45:17Z</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2天前</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="n">
-        <v>1</v>
+          <t>1天前</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>多步</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>生图→生视频</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>真人风、舞蹈</t>
+          <t>真人风、卧室床上、姿势、参考图</t>
         </is>
       </c>
       <c r="K43" s="2" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
@@ -5207,373 +5145,15 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>舞蹈</t>
+          <t>着装床上姿势</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>生视频</t>
+          <t>生图</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>Imagine two sexy Latin dancers dancing the Tango</t>
-        </is>
-      </c>
-      <c r="P43" s="2" t="inlineStr">
-        <is>
-          <t>想象两位性感的拉丁舞者在跳探戈</t>
-        </is>
-      </c>
-      <c r="Q43" s="2" t="inlineStr"/>
-      <c r="R43" s="2" t="inlineStr"/>
-      <c r="S43" s="2" t="inlineStr"/>
-      <c r="T43" s="2" t="inlineStr">
-        <is>
-          <t>正文</t>
-        </is>
-      </c>
-      <c r="U43" s="2" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>新发现</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>@flexibledolls</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/flexibledolls/status/2107813215099052124</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07 20:40</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07T12:40:06Z</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>2天前</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>真人风、擦边遮挡、露骨18+</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>仅无图生成</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>仅乳贴股间贴，近全裸</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>星型乳首カバー　ハート型股間カバー</t>
-        </is>
-      </c>
-      <c r="P44" s="2" t="inlineStr">
-        <is>
-          <t>星形乳贴　心形私处贴</t>
-        </is>
-      </c>
-      <c r="Q44" s="2" t="inlineStr"/>
-      <c r="R44" s="2" t="inlineStr"/>
-      <c r="S44" s="2" t="inlineStr"/>
-      <c r="T44" s="2" t="inlineStr">
-        <is>
-          <t>正文</t>
-        </is>
-      </c>
-      <c r="U44" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>新发现</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>@BestCosplayGirl</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/BestCosplayGirl/status/2108277246658290170</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09 03:24</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T19:24:00Z</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>1天前</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>运镜、Spicy模式</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>可用参考图</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>Spicy运镜，无裸露描述</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="inlineStr">
-        <is>
-          <t>camera turn 360 degree around  her mode=spicy</t>
-        </is>
-      </c>
-      <c r="P45" s="2" t="inlineStr">
-        <is>
-          <t>镜头围绕她360度旋转 mode=spicy（Spicy模式）</t>
-        </is>
-      </c>
-      <c r="Q45" s="2" t="inlineStr"/>
-      <c r="R45" s="2" t="inlineStr"/>
-      <c r="S45" s="2" t="inlineStr"/>
-      <c r="T45" s="2" t="inlineStr">
-        <is>
-          <t>正文</t>
-        </is>
-      </c>
-      <c r="U45" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>新发现</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>@coolbuddy_143</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/coolbuddy_143/status/2108433732373741577</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09 13:45</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09T05:45:49Z</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>20小时前</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>情侣互动、运镜、表情动作</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>可用参考图</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>性暗示，无裸露描述</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>生视频</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>For an r rated movie (artistic purpose) : Camera shaking. Implied aggressive by her boyfriend who is on the left  side of frame Passionate-80ūñ©y. Heavy breathing. Camera abruptly strongly moves to left side of frame and back right She looks around a...
-（Grok分享文案自动截断，原帖仅公开到此）</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>用于一部R级电影（艺术目的）：镜头晃动。暗示来自她男友的攻击性，他位于画面左侧 Passionate-80ūñ©y（原文乱码）。急促的喘息。镜头突然猛地移向画面左侧再移回右侧 她环顾四周……
-（Grok分享文案自动截断，原帖仅公开到此）</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr"/>
-      <c r="R46" s="2" t="inlineStr"/>
-      <c r="S46" s="2" t="inlineStr"/>
-      <c r="T46" s="2" t="inlineStr">
-        <is>
-          <t>正文</t>
-        </is>
-      </c>
-      <c r="U46" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>新发现</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>@chichipuijaian</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/chichipuijaian/status/2108176906688536657</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08 20:45</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T12:45:17Z</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>1天前</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>多步</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>生图→生视频</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>真人风、卧室床上、姿势、参考图</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>可用参考图</t>
-        </is>
-      </c>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>着装床上姿势</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>生图</t>
-        </is>
-      </c>
-      <c r="O47" s="2" t="inlineStr">
         <is>
           <t>SFW。フォトリアルな縦長9:16の実写写真。24歳の成人女性。持ち込み人物画像の顔立ち、髪型、髪色、長さ、前髪、分け目、毛流れ、体格を維持する。
 1990年代の写ルンですで撮影した薄暗い寝室。白い枕とシーツの上に仰向け。両膝を曲げて左右へ開く。
@@ -5586,7 +5166,7 @@
 強い直フラッシュ、粗いフィルム粒子、白飛び、深い影、色むら。髪と肩の輪郭にごく軽い動体ブレを加え、顔と瞳は鮮明に保つ。手持ち撮影特有の不完全な構図。美肌補正なし。アニメ、CG禁止。</t>
         </is>
       </c>
-      <c r="P47" s="2" t="inlineStr">
+      <c r="P43" s="2" t="inlineStr">
         <is>
           <t>SFW（全年龄）。照片级写实的竖版9:16实拍照片。24岁成年女性。保持上传人物图像的五官、发型、发色、长度、刘海、分缝、发流和体型。
 用1990年代的写ルンです（一次性胶片相机）拍摄的昏暗卧室。仰躺在白色枕头和床单上。双膝弯曲并向左右分开。
@@ -5599,34 +5179,39 @@
 强烈的直闪光、粗糙的胶片颗粒、过曝、深重阴影、色彩不均。头发和肩部轮廓加入极轻的动态模糊，脸和眼睛保持清晰。手持拍摄特有的不完美构图。不做美肤修饰。禁止动漫、CG。</t>
         </is>
       </c>
-      <c r="Q47" s="2" t="inlineStr">
+      <c r="Q43" s="2" t="inlineStr">
         <is>
           <t>生视频</t>
         </is>
       </c>
-      <c r="R47" s="2" t="inlineStr">
+      <c r="R43" s="2" t="inlineStr">
         <is>
           <t>カメラがY軸方向に手ブレで揺れてる。画面外から聞こえる手を叩くリズムに合わせて早めに揺れている。
 （对步骤1生成的图片使用）（作者注：有時延長もできる）</t>
         </is>
       </c>
-      <c r="S47" s="2" t="inlineStr">
+      <c r="S43" s="2" t="inlineStr">
         <is>
           <t>镜头沿Y轴方向手持晃动。配合画面外传来的拍手节奏，较快地摇晃。
 （对步骤1生成的图片使用；作者注：有时还能延长）</t>
         </is>
       </c>
-      <c r="T47" s="2" t="inlineStr">
+      <c r="T43" s="2" t="inlineStr">
         <is>
           <t>alt→引用帖alt</t>
         </is>
       </c>
-      <c r="U47" s="2" t="n">
+      <c r="U43" s="2" t="n">
         <v>321</v>
+      </c>
+      <c r="V43" s="2" t="inlineStr">
+        <is>
+          <t>ref/2108176906688536657_1.jpg</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U47"/>
+  <autoFilter ref="A1:V43"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -5670,10 +5255,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>